<commit_message>
Verify Blue Goat under-$200 picks against Semrush backlinks
Checked all 26 picks for existing links to bluegoatcyber.com. coruzant.com
had a live dofollow link (Ahrefs missed it) - removed. Remaining 25 confirmed
not-built on Semrush. Added verification column.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EyZhZSnP6QyNR5y5EJdqhU
</commit_message>
<xml_diff>
--- a/bluegoatcyber-under200-picks.xlsx
+++ b/bluegoatcyber-under200-picks.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:J26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -435,6 +435,7 @@
     <col width="9" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -483,6 +484,11 @@
           <t>Fit note</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Semrush check</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -518,6 +524,11 @@
           <t>★★ dev community, best value</t>
         </is>
       </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>NOT built (verified)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -533,7 +544,6 @@
       <c r="C3" t="n">
         <v>54</v>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="n">
         <v>35</v>
       </c>
@@ -551,6 +561,11 @@
           <t>docs platform - branded anchor</t>
         </is>
       </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>NOT built (verified)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -566,7 +581,6 @@
       <c r="C4" t="n">
         <v>51</v>
       </c>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="n">
         <v>27</v>
       </c>
@@ -584,779 +598,847 @@
           <t>tech courses/education</t>
         </is>
       </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>NOT built (verified)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>coruzant.com</t>
+          <t>strikingly.com</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Business-Tech</t>
+          <t>Web(UGC)</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>50</v>
-      </c>
-      <c r="D5" t="inlineStr"/>
+        <v>49</v>
+      </c>
       <c r="E5" t="n">
-        <v>26</v>
+        <v>45</v>
       </c>
       <c r="F5" t="n">
-        <v>210038</v>
+        <v>75229</v>
       </c>
       <c r="G5" t="n">
-        <v>95</v>
+        <v>55</v>
       </c>
       <c r="H5" t="n">
-        <v>10077</v>
+        <v>77701</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>business/tech interviews</t>
+          <t>site builder - branded anchor</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>NOT built (verified)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>strikingly.com</t>
+          <t>electronicsforu.com</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Web(UGC)</t>
+          <t>Electronics</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>49</v>
-      </c>
-      <c r="D6" t="inlineStr"/>
+        <v>48</v>
+      </c>
+      <c r="D6" t="n">
+        <v>47</v>
+      </c>
       <c r="E6" t="n">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="F6" t="n">
-        <v>75229</v>
+        <v>125324</v>
       </c>
       <c r="G6" t="n">
-        <v>55</v>
+        <v>110</v>
       </c>
       <c r="H6" t="n">
-        <v>77701</v>
+        <v>8465</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>site builder - branded anchor</t>
+          <t>★ electronics/devices news</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>NOT built (verified)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>electronicsforu.com</t>
+          <t>rapidapi.com</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Electronics</t>
+          <t>API/Dev</t>
         </is>
       </c>
       <c r="C7" t="n">
         <v>48</v>
       </c>
-      <c r="D7" t="n">
-        <v>47</v>
-      </c>
       <c r="E7" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F7" t="n">
-        <v>125324</v>
+        <v>194063</v>
       </c>
       <c r="G7" t="n">
-        <v>110</v>
+        <v>165</v>
       </c>
       <c r="H7" t="n">
-        <v>8465</v>
+        <v>52353</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>★ electronics/devices news</t>
+          <t>API/developer platform</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>NOT built (verified)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>rapidapi.com</t>
+          <t>gitbook.com</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>API/Dev</t>
+          <t>Dev-Tools</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>48</v>
-      </c>
-      <c r="D8" t="inlineStr"/>
+        <v>46</v>
+      </c>
+      <c r="D8" t="n">
+        <v>55</v>
+      </c>
       <c r="E8" t="n">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="F8" t="n">
-        <v>194063</v>
+        <v>90146</v>
       </c>
       <c r="G8" t="n">
-        <v>165</v>
+        <v>110</v>
       </c>
       <c r="H8" t="n">
-        <v>52353</v>
+        <v>59330</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>API/developer platform</t>
+          <t>developer docs/tools</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>NOT built (verified)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>gitbook.com</t>
+          <t>techimply.com</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Dev-Tools</t>
+          <t>SaaS/Web</t>
         </is>
       </c>
       <c r="C9" t="n">
         <v>46</v>
       </c>
-      <c r="D9" t="n">
-        <v>55</v>
-      </c>
       <c r="E9" t="n">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="F9" t="n">
-        <v>90146</v>
+        <v>28065</v>
       </c>
       <c r="G9" t="n">
-        <v>110</v>
+        <v>99</v>
       </c>
       <c r="H9" t="n">
-        <v>59330</v>
+        <v>4955</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>developer docs/tools</t>
+          <t>web dev/software reviews</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>NOT built (verified)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>techimply.com</t>
+          <t>hashnode.com</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>SaaS/Web</t>
+          <t>Dev</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>46</v>
-      </c>
-      <c r="D10" t="inlineStr"/>
+        <v>45</v>
+      </c>
       <c r="E10" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="F10" t="n">
-        <v>28065</v>
+        <v>79691</v>
       </c>
       <c r="G10" t="n">
-        <v>99</v>
+        <v>112</v>
       </c>
       <c r="H10" t="n">
-        <v>4955</v>
+        <v>83442</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>web dev/software reviews</t>
+          <t>developer blogging (SaaS)</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>NOT built (verified)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>hashnode.com</t>
+          <t>aijourn.com</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Dev</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>45</v>
-      </c>
-      <c r="D11" t="inlineStr"/>
+        <v>43</v>
+      </c>
+      <c r="D11" t="n">
+        <v>44</v>
+      </c>
       <c r="E11" t="n">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="F11" t="n">
-        <v>79691</v>
+        <v>91117</v>
       </c>
       <c r="G11" t="n">
-        <v>112</v>
+        <v>140</v>
       </c>
       <c r="H11" t="n">
-        <v>83442</v>
+        <v>14059</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>developer blogging (SaaS)</t>
+          <t>AI news/research</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>NOT built (verified)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>aijourn.com</t>
+          <t>theengineeringprojects.com</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="C12" t="n">
+        <v>42</v>
+      </c>
+      <c r="D12" t="n">
         <v>43</v>
       </c>
-      <c r="D12" t="n">
-        <v>44</v>
-      </c>
       <c r="E12" t="n">
-        <v>40</v>
+        <v>22</v>
       </c>
       <c r="F12" t="n">
-        <v>91117</v>
+        <v>83472</v>
       </c>
       <c r="G12" t="n">
-        <v>140</v>
+        <v>190</v>
       </c>
       <c r="H12" t="n">
-        <v>14059</v>
+        <v>4386</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>AI news/research</t>
+          <t>★ embedded/engineering</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>NOT built (verified)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>theengineeringprojects.com</t>
+          <t>ijert.org</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>Eng-Research</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D13" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="E13" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F13" t="n">
-        <v>83472</v>
+        <v>26869</v>
       </c>
       <c r="G13" t="n">
-        <v>190</v>
+        <v>140</v>
       </c>
       <c r="H13" t="n">
-        <v>4386</v>
+        <v>5660</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>★ embedded/engineering</t>
+          <t>engineering research journal</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>NOT built (verified)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ijert.org</t>
+          <t>saasadviser.co</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Eng-Research</t>
+          <t>SaaS</t>
         </is>
       </c>
       <c r="C14" t="n">
         <v>41</v>
       </c>
-      <c r="D14" t="n">
-        <v>41</v>
-      </c>
       <c r="E14" t="n">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="F14" t="n">
-        <v>26869</v>
+        <v>71856</v>
       </c>
       <c r="G14" t="n">
         <v>140</v>
       </c>
       <c r="H14" t="n">
-        <v>5660</v>
+        <v>2931</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>engineering research journal</t>
+          <t>SaaS advisory</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>NOT built (verified)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>saasadviser.co</t>
+          <t>devopsschool.com</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>SaaS</t>
+          <t>DevOps</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>41</v>
-      </c>
-      <c r="D15" t="inlineStr"/>
+        <v>40</v>
+      </c>
       <c r="E15" t="n">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="F15" t="n">
-        <v>71856</v>
+        <v>30028</v>
       </c>
       <c r="G15" t="n">
-        <v>140</v>
+        <v>150</v>
       </c>
       <c r="H15" t="n">
-        <v>2931</v>
+        <v>3664</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>SaaS advisory</t>
+          <t>devops/training</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>NOT built (verified)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>devopsschool.com</t>
+          <t>excelforum.com</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>DevOps</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="C16" t="n">
         <v>40</v>
       </c>
-      <c r="D16" t="inlineStr"/>
       <c r="E16" t="n">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="F16" t="n">
-        <v>30028</v>
+        <v>35231</v>
       </c>
       <c r="G16" t="n">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="H16" t="n">
-        <v>3664</v>
+        <v>3951</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>devops/training</t>
+          <t>electronics/hardware forum</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>NOT built (verified)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>excelforum.com</t>
+          <t>enterpriseitworld.com</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>Enterprise-IT</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>40</v>
-      </c>
-      <c r="D17" t="inlineStr"/>
+        <v>37</v>
+      </c>
+      <c r="D17" t="n">
+        <v>38</v>
+      </c>
       <c r="E17" t="n">
-        <v>36</v>
+        <v>22</v>
       </c>
       <c r="F17" t="n">
-        <v>35231</v>
+        <v>21297</v>
       </c>
       <c r="G17" t="n">
-        <v>157</v>
+        <v>127</v>
       </c>
       <c r="H17" t="n">
-        <v>3951</v>
+        <v>1717</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>electronics/hardware forum</t>
+          <t>★ enterprise IT</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>NOT built (verified)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>enterpriseitworld.com</t>
+          <t>ourcodeworld.com</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Enterprise-IT</t>
+          <t>Programming</t>
         </is>
       </c>
       <c r="C18" t="n">
         <v>37</v>
       </c>
-      <c r="D18" t="n">
-        <v>38</v>
-      </c>
       <c r="E18" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F18" t="n">
-        <v>21297</v>
+        <v>16104</v>
       </c>
       <c r="G18" t="n">
-        <v>127</v>
+        <v>150</v>
       </c>
       <c r="H18" t="n">
-        <v>1717</v>
+        <v>3630</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>★ enterprise IT</t>
+          <t>programming/education</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>NOT built (verified)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ourcodeworld.com</t>
+          <t>content.techgig.com</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Programming</t>
+          <t>Dev</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>37</v>
-      </c>
-      <c r="D19" t="inlineStr"/>
+        <v>36</v>
+      </c>
       <c r="E19" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F19" t="n">
-        <v>16104</v>
+        <v>12160</v>
       </c>
       <c r="G19" t="n">
-        <v>150</v>
+        <v>165</v>
       </c>
       <c r="H19" t="n">
-        <v>3630</v>
+        <v>4044</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>programming/education</t>
+          <t>developer community</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>NOT built (verified)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>content.techgig.com</t>
+          <t>hardwaresecrets.com</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Dev</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>36</v>
-      </c>
-      <c r="D20" t="inlineStr"/>
+        <v>35</v>
+      </c>
       <c r="E20" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F20" t="n">
-        <v>12160</v>
+        <v>268641</v>
       </c>
       <c r="G20" t="n">
-        <v>165</v>
+        <v>150</v>
       </c>
       <c r="H20" t="n">
-        <v>4044</v>
+        <v>5326</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>developer community</t>
+          <t>hardware/electronics</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>NOT built (verified)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>hardwaresecrets.com</t>
+          <t>includehelp.com</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>Programming</t>
         </is>
       </c>
       <c r="C21" t="n">
         <v>35</v>
       </c>
-      <c r="D21" t="inlineStr"/>
       <c r="E21" t="n">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="F21" t="n">
-        <v>268641</v>
+        <v>20086</v>
       </c>
       <c r="G21" t="n">
         <v>150</v>
       </c>
       <c r="H21" t="n">
-        <v>5326</v>
+        <v>2096</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>hardware/electronics</t>
+          <t>programming tutorials</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>NOT built (verified)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>includehelp.com</t>
+          <t>ipwithease.com</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Programming</t>
+          <t>Networking/Security</t>
         </is>
       </c>
       <c r="C22" t="n">
+        <v>34</v>
+      </c>
+      <c r="D22" t="n">
         <v>35</v>
       </c>
-      <c r="D22" t="inlineStr"/>
       <c r="E22" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F22" t="n">
-        <v>20086</v>
+        <v>11606</v>
       </c>
       <c r="G22" t="n">
-        <v>150</v>
+        <v>60</v>
       </c>
       <c r="H22" t="n">
-        <v>2096</v>
+        <v>1316</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>programming tutorials</t>
+          <t>★ networking/security/cloud</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>NOT built (verified)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ipwithease.com</t>
+          <t>innovareacademics.in</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Networking/Security</t>
+          <t>Digital-Health</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>34</v>
-      </c>
-      <c r="D23" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="E23" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="F23" t="n">
-        <v>11606</v>
+        <v>10982</v>
       </c>
       <c r="G23" t="n">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="H23" t="n">
-        <v>1316</v>
+        <v>5736</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>★ networking/security/cloud</t>
+          <t>digital health/research</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>NOT built (verified)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>innovareacademics.in</t>
+          <t>clinicalgate.com</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Digital-Health</t>
+          <t>Medical-Ref</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>38</v>
-      </c>
-      <c r="D24" t="inlineStr"/>
+        <v>36</v>
+      </c>
+      <c r="D24" t="n">
+        <v>36</v>
+      </c>
       <c r="E24" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F24" t="n">
-        <v>10982</v>
+        <v>10428</v>
       </c>
       <c r="G24" t="n">
-        <v>90</v>
+        <v>175</v>
       </c>
       <c r="H24" t="n">
-        <v>5736</v>
+        <v>2729</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>digital health/research</t>
+          <t>★ clinical/medical reference</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>NOT built (verified)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>clinicalgate.com</t>
+          <t>psbios.com</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Medical-Ref</t>
+          <t>Bioscience</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>36</v>
-      </c>
-      <c r="D25" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E25" t="n">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="F25" t="n">
-        <v>10428</v>
+        <v>6803</v>
       </c>
       <c r="G25" t="n">
-        <v>175</v>
+        <v>15</v>
       </c>
       <c r="H25" t="n">
-        <v>2729</v>
+        <v>7133</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>★ clinical/medical reference</t>
+          <t>bioscience/research/tech, cheap</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>NOT built (verified)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>psbios.com</t>
+          <t>drugtodayonline.com</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Bioscience</t>
+          <t>Pharma</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>35</v>
-      </c>
-      <c r="D26" t="inlineStr"/>
+        <v>33</v>
+      </c>
       <c r="E26" t="n">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="F26" t="n">
-        <v>6803</v>
+        <v>5846</v>
       </c>
       <c r="G26" t="n">
-        <v>15</v>
+        <v>110</v>
       </c>
       <c r="H26" t="n">
-        <v>7133</v>
+        <v>1288</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>bioscience/research/tech, cheap</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>drugtodayonline.com</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Pharma</t>
-        </is>
-      </c>
-      <c r="C27" t="n">
-        <v>33</v>
-      </c>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="n">
-        <v>22</v>
-      </c>
-      <c r="F27" t="n">
-        <v>5846</v>
-      </c>
-      <c r="G27" t="n">
-        <v>110</v>
-      </c>
-      <c r="H27" t="n">
-        <v>1288</v>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
           <t>health/pharma news</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>NOT built (verified)</t>
         </is>
       </c>
     </row>

</xml_diff>